<commit_message>
Corrections to plat/prog and ECV/dtype mappings
</commit_message>
<xml_diff>
--- a/data/cci/cci-dataType-ecv-mapping.xlsx
+++ b/data/cci/cci-dataType-ecv-mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stfc365-my.sharepoint.com/personal/alison_waterfall_stfc_ac_uk/Documents/Documents/GitHub/cci-vocabularies/data/cci/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{988F0833-324E-A94E-ADCC-47810A45B928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9733AD3D-2347-4A42-A480-A10037525630}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{988F0833-324E-A94E-ADCC-47810A45B928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43199E8C-6F20-480D-A352-BAE349986048}"/>
   <bookViews>
-    <workbookView xWindow="9000" yWindow="2700" windowWidth="28800" windowHeight="15285" xr2:uid="{4E51E550-2BE2-1645-BA80-54EF4527885D}"/>
+    <workbookView xWindow="39450" yWindow="3285" windowWidth="34515" windowHeight="15285" xr2:uid="{4E51E550-2BE2-1645-BA80-54EF4527885D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -345,9 +345,6 @@
     <t>dtype_lst</t>
   </si>
   <si>
-    <t>cciecv_lst</t>
-  </si>
-  <si>
     <t>dtype_pft</t>
   </si>
   <si>
@@ -376,6 +373,9 @@
   </si>
   <si>
     <t>dtype_nh3</t>
+  </si>
+  <si>
+    <t>cciecv_landSurfTemp</t>
   </si>
 </sst>
 </file>
@@ -2175,7 +2175,7 @@
         <v>5</v>
       </c>
       <c r="C84" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="D84" t="s">
         <v>7</v>
@@ -2183,7 +2183,7 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B85" t="s">
         <v>5</v>
@@ -2197,7 +2197,7 @@
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B86" t="s">
         <v>5</v>
@@ -2211,13 +2211,13 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>108</v>
+      </c>
+      <c r="B87" t="s">
+        <v>5</v>
+      </c>
+      <c r="C87" t="s">
         <v>109</v>
-      </c>
-      <c r="B87" t="s">
-        <v>5</v>
-      </c>
-      <c r="C87" t="s">
-        <v>110</v>
       </c>
       <c r="D87" t="s">
         <v>7</v>
@@ -2225,13 +2225,13 @@
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>110</v>
+      </c>
+      <c r="B88" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" t="s">
         <v>111</v>
-      </c>
-      <c r="B88" t="s">
-        <v>5</v>
-      </c>
-      <c r="C88" t="s">
-        <v>112</v>
       </c>
       <c r="D88" t="s">
         <v>7</v>
@@ -2239,7 +2239,7 @@
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B89" t="s">
         <v>5</v>
@@ -2253,13 +2253,13 @@
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>114</v>
+      </c>
+      <c r="B90" t="s">
+        <v>5</v>
+      </c>
+      <c r="C90" t="s">
         <v>115</v>
-      </c>
-      <c r="B90" t="s">
-        <v>5</v>
-      </c>
-      <c r="C90" t="s">
-        <v>116</v>
       </c>
       <c r="D90" t="s">
         <v>7</v>
@@ -2267,13 +2267,13 @@
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B91" t="s">
         <v>5</v>
       </c>
       <c r="C91" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D91" t="s">
         <v>7</v>

</xml_diff>